<commit_message>
Add daily reflections for October, November, and December, along with README and application voice logic documentation
- Created daily reflections for October (30 entries), November (30 entries), and December (31 entries) focusing on themes of meaning, gratitude, and sharing.
- Added a README file outlining the structure and purpose of the daily reflections.
- Introduced a document detailing the voice logic of the application, emphasizing user-friendliness and supportive communication.
</commit_message>
<xml_diff>
--- a/docs/codzienne-refleksje-plan.xlsx
+++ b/docs/codzienne-refleksje-plan.xlsx
@@ -169,7 +169,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moment, w ktorym przestajesz uciekac</t>
+          <t xml:space="preserve">Przestaje uciekac</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -247,7 +247,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cisza, ktora zaczyna mowic</t>
+          <t xml:space="preserve">W ciszy zaczynam slyszec</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
@@ -325,7 +325,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pierwsza uczciwosc wobec siebie</t>
+          <t xml:space="preserve">Mowie sobie prawde</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -403,7 +403,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kiedy juz nie da sie udawac</t>
+          <t xml:space="preserve">Przestaje udawac</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -481,7 +481,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zmeczenie zyciem w napieciu</t>
+          <t xml:space="preserve">Rozpoznaje swoje zmeczenie</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
@@ -559,7 +559,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prawda pojawia sie powoli</t>
+          <t xml:space="preserve">Daje sobie czas</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -637,7 +637,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zatrzymac sie, zeby zobaczyc</t>
+          <t xml:space="preserve">Zatrzymuje sie, zeby zobaczyc</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -715,7 +715,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzien, w ktorym cos peka</t>
+          <t xml:space="preserve">Widze, ze cos we mnie peka</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
@@ -793,7 +793,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kiedy przestajesz walczyc z rzeczywistoscia</t>
+          <t xml:space="preserve">Przestaje walczyc z rzeczywistoscia</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -871,7 +871,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pierwszy oddech bez iluzji</t>
+          <t xml:space="preserve">Biore pierwszy oddech bez iluzji</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -949,7 +949,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pomiedzy chaosem a nadzieja</t>
+          <t xml:space="preserve">Jestem pomiedzy chaosem a nadzieja</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -1027,7 +1027,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nie wiem co dalej</t>
+          <t xml:space="preserve">Nie wiem jeszcze co dalej</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -1105,7 +1105,7 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Przyznanie sie do bezradnosci</t>
+          <t xml:space="preserve">Przyznaje sie do bezradnosci</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Punkt, w ktorym koncza sie wymowki</t>
+          <t xml:space="preserve">Dochodze do punktu, w ktorym koncza sie wymowki</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kiedy zaczynasz slyszec siebie</t>
+          <t xml:space="preserve">Zaczynam slyszec siebie</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zatrzymanie to nie porazka</t>
+          <t xml:space="preserve">Widze, ze zatrzymanie to nie porazka</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
@@ -1417,7 +1417,7 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prawda o zmeczeniu</t>
+          <t xml:space="preserve">Widze prawde o swoim zmeczeniu</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
@@ -1495,7 +1495,7 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spotkanie z wlasnym zyciem</t>
+          <t xml:space="preserve">Spotykam sie z wlasnym zyciem</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
@@ -1573,7 +1573,7 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t xml:space="preserve">Przestac udawac sile</t>
+          <t xml:space="preserve">Przestaje udawac sile</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
@@ -1651,7 +1651,7 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t xml:space="preserve">Poczatek drogi zaczyna sie od prawdy</t>
+          <t xml:space="preserve">Zaczynam droge od prawdy</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1729,7 +1729,7 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gdy cisza staje sie lustrem</t>
+          <t xml:space="preserve">W ciszy widze siebie jak w lustrze</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1807,7 +1807,7 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nie wszystko da sie kontrolowac</t>
+          <t xml:space="preserve">Przyjmuje, ze nie wszystko moge kontrolowac</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1885,7 +1885,7 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t xml:space="preserve">Moment, w ktorym pojawia sie pokora</t>
+          <t xml:space="preserve">Ucze sie pokory</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1963,7 +1963,7 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zgoda na to, ze potrzebuje pomocy</t>
+          <t xml:space="preserve">Zgadzam sie na to, ze potrzebuje pomocy</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
@@ -2041,7 +2041,7 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wreszcie przestac udowadniac</t>
+          <t xml:space="preserve">Wreszcie przestaje udowadniac</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
@@ -2119,7 +2119,7 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pierwsza szczelina w murze</t>
+          <t xml:space="preserve">Widze pierwsza szczeline w murze</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
@@ -2197,7 +2197,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prawda nie musi byc wygodna</t>
+          <t xml:space="preserve">Przyjmuje, ze prawda nie musi byc wygodna</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -2275,7 +2275,7 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kiedy zaczynasz widziec konsekwencje</t>
+          <t xml:space="preserve">Zaczynam widziec konsekwencje</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
@@ -2353,7 +2353,7 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t xml:space="preserve">Uznanie wlasnej kruchosci</t>
+          <t xml:space="preserve">Uznaje wlasna kruchosc</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
@@ -2431,7 +2431,7 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Poczatek odpowiedzialnosci</t>
+          <t xml:space="preserve">Zaczynam brac odpowiedzialnosc</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
@@ -2509,7 +2509,7 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nowy rok w prawdzie</t>
+          <t xml:space="preserve">Wchodze w nowy rok w prawdzie</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
@@ -2587,7 +2587,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emocje, ktore wracaja</t>
+          <t xml:space="preserve">Emocje do mnie wracaja</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -2665,7 +2665,7 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zlosc, ktora chce byc uslyszana</t>
+          <t xml:space="preserve">Slucham swojej zlosci</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -2743,7 +2743,7 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smutek, ktory potrzebuje miejsca</t>
+          <t xml:space="preserve">Daje miejsce swojemu smutkowi</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
@@ -2821,7 +2821,7 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t xml:space="preserve">Strach, ktory probuje cie chronic</t>
+          <t xml:space="preserve">Widze strach, ktory probuje mnie chronic</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
@@ -2899,7 +2899,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wstyd, ktory zamyka drzwi</t>
+          <t xml:space="preserve">Widze wstyd, ktory zamyka mnie od srodka</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
@@ -2977,7 +2977,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t xml:space="preserve">Poczucie winy i odpowiedzialnosc</t>
+          <t xml:space="preserve">Rozrozniam poczucie winy i odpowiedzialnosc</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -3055,7 +3055,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t xml:space="preserve">Samotnosc w tlumie</t>
+          <t xml:space="preserve">Czuje samotnosc w tlumie</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
@@ -3133,7 +3133,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t xml:space="preserve">Radosc, ktora czasem oniesmiela</t>
+          <t xml:space="preserve">Otwieram sie na radosc</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
@@ -3211,7 +3211,7 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emocje sa informacja</t>
+          <t xml:space="preserve">Traktuje emocje jak informacje</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
@@ -3289,7 +3289,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kiedy uczucia zaczynaja wracac</t>
+          <t xml:space="preserve">Czuje, jak uczucia zaczynaja wracac</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -3367,7 +3367,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zlosc nie jest wrogiem</t>
+          <t xml:space="preserve">Przestaje walczyc ze swoja zloscia</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -3445,7 +3445,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t xml:space="preserve">Strach nie musi prowadzic</t>
+          <t xml:space="preserve">Nie pozwalam, by strach mnie prowadzil</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -3523,7 +3523,7 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smutek potrafi leczyc</t>
+          <t xml:space="preserve">Pozwalam smutkowi leczyc</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
@@ -3601,7 +3601,7 @@
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wstyd chce zostac zobaczony</t>
+          <t xml:space="preserve">Pozwalam zobaczyc swoj wstyd</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t xml:space="preserve">Poczucie winy moze prowadzic do zmiany</t>
+          <t xml:space="preserve">Pozwalam, by poczucie winy prowadzilo mnie do zmiany</t>
         </is>
       </c>
       <c r="G47" t="inlineStr">
@@ -3757,7 +3757,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t xml:space="preserve">Samotnosc moze byc poczatkiem spotkania</t>
+          <t xml:space="preserve">Odkrywam, ze samotnosc moze byc poczatkiem spotkania</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
@@ -3835,7 +3835,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t xml:space="preserve">Radosc jako odwaga zycia</t>
+          <t xml:space="preserve">Traktuje radosc jak odwage zycia</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
@@ -3913,7 +3913,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t xml:space="preserve">Emocje sa drogowskazem</t>
+          <t xml:space="preserve">Odczytuje emocje jak drogowskaz</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
@@ -3991,7 +3991,7 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t xml:space="preserve">Uczucia nie sa problemem</t>
+          <t xml:space="preserve">Przestaje traktowac uczucia jak problem</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -4069,7 +4069,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kiedy uczucia przestaja byc zagrozeniem</t>
+          <t xml:space="preserve">Uczucia przestaja byc dla mnie zagrozeniem</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -4147,7 +4147,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nauka nazywania emocji</t>
+          <t xml:space="preserve">Ucze sie nazywac emocje</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -4225,7 +4225,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kiedy przestajesz sie ich bac</t>
+          <t xml:space="preserve">Przestaje sie ich bac</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
@@ -4303,7 +4303,7 @@
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t xml:space="preserve">Uczucia jako jezyk zycia</t>
+          <t xml:space="preserve">Odczytuje uczucia jak jezyk zycia</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
@@ -4381,7 +4381,7 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zlosc mowi o granicach</t>
+          <t xml:space="preserve">Slysze, co moja zlosc mowi o granicach</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -4459,7 +4459,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t xml:space="preserve">Smutek mowi o stracie</t>
+          <t xml:space="preserve">Slysze, co moj smutek mowi o stracie</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
@@ -4537,7 +4537,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t xml:space="preserve">Strach mowi o niepewnosci</t>
+          <t xml:space="preserve">Slysze, co moj strach mowi o niepewnosci</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -4615,7 +4615,7 @@
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wstyd mowi o ukrywaniu</t>
+          <t xml:space="preserve">Slysze, co moj wstyd mowi o ukrywaniu</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
@@ -4693,7 +4693,7 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t xml:space="preserve">Poczucie winy mowi o odpowiedzialnosci</t>
+          <t xml:space="preserve">Slysze, co moje poczucie winy mowi o odpowiedzialnosci</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -4771,7 +4771,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzien dodatkowy: lagodnosc wobec siebie</t>
+          <t xml:space="preserve">Ucze sie lagodnosci wobec siebie</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
@@ -4849,7 +4849,7 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t xml:space="preserve">Historia, ktora sobie opowiadalem</t>
+          <t xml:space="preserve">Widze historie, ktora sobie opowiadam</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
@@ -4927,7 +4927,7 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mechanizmy obronne</t>
+          <t xml:space="preserve">Rozpoznaje swoje mechanizmy obronne</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -5005,7 +5005,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t xml:space="preserve">Racjonalizacje</t>
+          <t xml:space="preserve">Rozpoznaje swoje racjonalizacje</t>
         </is>
       </c>
       <c r="G64" t="inlineStr">
@@ -5083,7 +5083,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zaprzeczanie</t>
+          <t xml:space="preserve">Widze swoje zaprzeczanie</t>
         </is>
       </c>
       <c r="G65" t="inlineStr">
@@ -5161,7 +5161,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t xml:space="preserve">Minimalizowanie</t>
+          <t xml:space="preserve">Widze, jak minimalizuje</t>
         </is>
       </c>
       <c r="G66" t="inlineStr">
@@ -5239,7 +5239,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t xml:space="preserve">Przerzucanie winy</t>
+          <t xml:space="preserve">Przestaje przerzucac wine</t>
         </is>
       </c>
       <c r="G67" t="inlineStr">
@@ -5317,7 +5317,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ucieczka w kontrole</t>
+          <t xml:space="preserve">Uciekam w kontrole</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -5395,7 +5395,7 @@
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t xml:space="preserve">Ucieczka w chaos</t>
+          <t xml:space="preserve">Uciekam w chaos</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -5473,7 +5473,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t xml:space="preserve">Iluzja sily</t>
+          <t xml:space="preserve">Widze iluzje swojej sily</t>
         </is>
       </c>
       <c r="G70" t="inlineStr">
@@ -5551,7 +5551,7 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t xml:space="preserve">Iluzja wyjatkowosci</t>
+          <t xml:space="preserve">Widze iluzje swojej wyjatkowosci</t>
         </is>
       </c>
       <c r="G71" t="inlineStr">
@@ -5629,7 +5629,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t xml:space="preserve">Iluzja niewinnosci</t>
+          <t xml:space="preserve">Widze iluzje swojej niewinnosci</t>
         </is>
       </c>
       <c r="G72" t="inlineStr">
@@ -5707,7 +5707,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kiedy zaczynasz widziec schemat</t>
+          <t xml:space="preserve">Zaczynam widziec schemat</t>
         </is>
       </c>
       <c r="G73" t="inlineStr">
@@ -5785,7 +5785,7 @@
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odkrywanie wlasnych manipulacji</t>
+          <t xml:space="preserve">Odkrywam swoje manipulacje</t>
         </is>
       </c>
       <c r="G74" t="inlineStr">
@@ -5863,7 +5863,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t xml:space="preserve">Historia, ktora budowalem o sobie</t>
+          <t xml:space="preserve">Widze historie, ktora buduje o sobie</t>
         </is>
       </c>
       <c r="G75" t="inlineStr">
@@ -5941,7 +5941,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prawda o mojej roli</t>
+          <t xml:space="preserve">Widze prawde o swojej roli</t>
         </is>
       </c>
       <c r="G76" t="inlineStr">
@@ -6019,7 +6019,7 @@
       </c>
       <c r="F77" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mechanizmy, ktore mnie chronily</t>
+          <t xml:space="preserve">Widze mechanizmy, ktore mnie chronily</t>
         </is>
       </c>
       <c r="G77" t="inlineStr">
@@ -6097,7 +6097,7 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kiedy obrona staje sie wiezieniem</t>
+          <t xml:space="preserve">Widze, kiedy obrona staje sie wiezieniem</t>
         </is>
       </c>
       <c r="G78" t="inlineStr">
@@ -6175,7 +6175,7 @@
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zobaczyc swoje strategie</t>
+          <t xml:space="preserve">Zaczynam widziec swoje strategie</t>
         </is>
       </c>
       <c r="G79" t="inlineStr">
@@ -6253,7 +6253,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t xml:space="preserve">Przestac walczyc z rzeczywistoscia</t>
+          <t xml:space="preserve">Przestaje walczyc z rzeczywistoscia</t>
         </is>
       </c>
       <c r="G80" t="inlineStr">
@@ -6331,7 +6331,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zrozumiec wlasne klamstwa</t>
+          <t xml:space="preserve">Zaczynam rozumiec swoje klamstwa</t>
         </is>
       </c>
       <c r="G81" t="inlineStr">
@@ -6409,7 +6409,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kiedy zaczyna sie uczciwosc</t>
+          <t xml:space="preserve">Zaczynam byc uczciwy</t>
         </is>
       </c>
       <c r="G82" t="inlineStr">
@@ -6487,7 +6487,7 @@
       </c>
       <c r="F83" t="inlineStr">
         <is>
-          <t xml:space="preserve">Widziec bez usprawiedliwien</t>
+          <t xml:space="preserve">Widze bez usprawiedliwien</t>
         </is>
       </c>
       <c r="G83" t="inlineStr">
@@ -6565,7 +6565,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t xml:space="preserve">Konfrontacja z prawda</t>
+          <t xml:space="preserve">Konfrontuje sie z prawda</t>
         </is>
       </c>
       <c r="G84" t="inlineStr">
@@ -6643,7 +6643,7 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t xml:space="preserve">Iluzja kontroli</t>
+          <t xml:space="preserve">Widze iluzje kontroli</t>
         </is>
       </c>
       <c r="G85" t="inlineStr">
@@ -6721,7 +6721,7 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t xml:space="preserve">Iluzja bezpieczenstwa</t>
+          <t xml:space="preserve">Widze iluzje bezpieczenstwa</t>
         </is>
       </c>
       <c r="G86" t="inlineStr">
@@ -6799,7 +6799,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t xml:space="preserve">Iluzja samotnosci</t>
+          <t xml:space="preserve">Widze iluzje samotnosci</t>
         </is>
       </c>
       <c r="G87" t="inlineStr">
@@ -6877,7 +6877,7 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t xml:space="preserve">Iluzja samowystarczalnosci</t>
+          <t xml:space="preserve">Widze iluzje samowystarczalnosci</t>
         </is>
       </c>
       <c r="G88" t="inlineStr">
@@ -6955,7 +6955,7 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t xml:space="preserve">Iluzja niezaleznosci</t>
+          <t xml:space="preserve">Widze iluzje niezaleznosci</t>
         </is>
       </c>
       <c r="G89" t="inlineStr">
@@ -7033,7 +7033,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t xml:space="preserve">Iluzja wyjatkowego cierpienia</t>
+          <t xml:space="preserve">Widze iluzje wyjatkowego cierpienia</t>
         </is>
       </c>
       <c r="G90" t="inlineStr">
@@ -7111,7 +7111,7 @@
       </c>
       <c r="F91" t="inlineStr">
         <is>
-          <t xml:space="preserve">Iluzja, ze jestem inny</t>
+          <t xml:space="preserve">Przestaje wierzyc, ze jestem inny</t>
         </is>
       </c>
       <c r="G91" t="inlineStr">
@@ -7189,7 +7189,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t xml:space="preserve">Poczatek trzezwego widzenia</t>
+          <t xml:space="preserve">Zaczynam widziec trzezwo</t>
         </is>
       </c>
       <c r="G92" t="inlineStr">
@@ -7267,7 +7267,7 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za swoje zycie</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za swoje zycie</t>
         </is>
       </c>
       <c r="G93" t="inlineStr">
@@ -7345,7 +7345,7 @@
       </c>
       <c r="F94" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za swoje decyzje</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za swoje decyzje</t>
         </is>
       </c>
       <c r="G94" t="inlineStr">
@@ -7423,7 +7423,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za swoje emocje</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za swoje emocje</t>
         </is>
       </c>
       <c r="G95" t="inlineStr">
@@ -7501,7 +7501,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za swoje slowa</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za swoje slowa</t>
         </is>
       </c>
       <c r="G96" t="inlineStr">
@@ -7579,7 +7579,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za relacje</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za relacje</t>
         </is>
       </c>
       <c r="G97" t="inlineStr">
@@ -7657,7 +7657,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za granice</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za granice</t>
         </is>
       </c>
       <c r="G98" t="inlineStr">
@@ -7735,7 +7735,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za zmiany</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za zmiany</t>
         </is>
       </c>
       <c r="G99" t="inlineStr">
@@ -7813,7 +7813,7 @@
       </c>
       <c r="F100" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za prawde</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za prawde</t>
         </is>
       </c>
       <c r="G100" t="inlineStr">
@@ -7891,7 +7891,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za konsekwencje</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za konsekwencje</t>
         </is>
       </c>
       <c r="G101" t="inlineStr">
@@ -7969,7 +7969,7 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za wybory</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za wybory</t>
         </is>
       </c>
       <c r="G102" t="inlineStr">
@@ -8047,7 +8047,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za przeszlosc</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za przeszlosc</t>
         </is>
       </c>
       <c r="G103" t="inlineStr">
@@ -8125,7 +8125,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za przyszlosc</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za przyszlosc</t>
         </is>
       </c>
       <c r="G104" t="inlineStr">
@@ -8203,7 +8203,7 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za dzien dzisiejszy</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za dzien dzisiejszy</t>
         </is>
       </c>
       <c r="G105" t="inlineStr">
@@ -8281,7 +8281,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za uczciwosc</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za uczciwosc</t>
         </is>
       </c>
       <c r="G106" t="inlineStr">
@@ -8359,7 +8359,7 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za bledy</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za bledy</t>
         </is>
       </c>
       <c r="G107" t="inlineStr">
@@ -8437,7 +8437,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za naprawe</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za naprawe</t>
         </is>
       </c>
       <c r="G108" t="inlineStr">
@@ -8515,7 +8515,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za sluchanie</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za sluchanie</t>
         </is>
       </c>
       <c r="G109" t="inlineStr">
@@ -8593,7 +8593,7 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za milczenie</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za milczenie</t>
         </is>
       </c>
       <c r="G110" t="inlineStr">
@@ -8671,7 +8671,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za dzialanie</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za dzialanie</t>
         </is>
       </c>
       <c r="G111" t="inlineStr">
@@ -8749,7 +8749,7 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za relacje z samym soba</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za relacje z samym soba</t>
         </is>
       </c>
       <c r="G112" t="inlineStr">
@@ -8827,7 +8827,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za cialo</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za cialo</t>
         </is>
       </c>
       <c r="G113" t="inlineStr">
@@ -8905,7 +8905,7 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za czas</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za czas</t>
         </is>
       </c>
       <c r="G114" t="inlineStr">
@@ -8983,7 +8983,7 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za rozwoj</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za rozwoj</t>
         </is>
       </c>
       <c r="G115" t="inlineStr">
@@ -9061,7 +9061,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za pomoc</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za pomoc</t>
         </is>
       </c>
       <c r="G116" t="inlineStr">
@@ -9139,7 +9139,7 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za przyjecie pomocy</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za przyjecie pomocy</t>
         </is>
       </c>
       <c r="G117" t="inlineStr">
@@ -9217,7 +9217,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za zmiane</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za zmiane</t>
         </is>
       </c>
       <c r="G118" t="inlineStr">
@@ -9295,7 +9295,7 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za prawde o sobie</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za prawde o sobie</t>
         </is>
       </c>
       <c r="G119" t="inlineStr">
@@ -9373,7 +9373,7 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za terazniejszosc</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za terazniejszosc</t>
         </is>
       </c>
       <c r="G120" t="inlineStr">
@@ -9451,7 +9451,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za droge</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za droge</t>
         </is>
       </c>
       <c r="G121" t="inlineStr">
@@ -9529,7 +9529,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc jako wolnosc</t>
+          <t xml:space="preserve">Odkrywam odpowiedzialnosc jako wolnosc</t>
         </is>
       </c>
       <c r="G122" t="inlineStr">
@@ -9607,7 +9607,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t xml:space="preserve">Relacje zaczynaja sie od prawdy</t>
+          <t xml:space="preserve">Zaczynam relacje od prawdy</t>
         </is>
       </c>
       <c r="G123" t="inlineStr">
@@ -9685,7 +9685,7 @@
       </c>
       <c r="F124" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spotkanie dwoch swiatow</t>
+          <t xml:space="preserve">Spotykam drugi swiat</t>
         </is>
       </c>
       <c r="G124" t="inlineStr">
@@ -9763,7 +9763,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kiedy zaczynam sluchac</t>
+          <t xml:space="preserve">Zaczynam sluchac</t>
         </is>
       </c>
       <c r="G125" t="inlineStr">
@@ -9841,7 +9841,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t xml:space="preserve">Relacja to nie kontrola</t>
+          <t xml:space="preserve">Widze, ze relacja to nie kontrola</t>
         </is>
       </c>
       <c r="G126" t="inlineStr">
@@ -9919,7 +9919,7 @@
       </c>
       <c r="F127" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bliskosc bez udawania</t>
+          <t xml:space="preserve">Ucze sie bliskosci bez udawania</t>
         </is>
       </c>
       <c r="G127" t="inlineStr">
@@ -9997,7 +9997,7 @@
       </c>
       <c r="F128" t="inlineStr">
         <is>
-          <t xml:space="preserve">Uwaznosc na drugiego czlowieka</t>
+          <t xml:space="preserve">Uwazam na drugiego czlowieka</t>
         </is>
       </c>
       <c r="G128" t="inlineStr">
@@ -10075,7 +10075,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mowic i byc slyszanym</t>
+          <t xml:space="preserve">Mowie i daje sie uslyszec</t>
         </is>
       </c>
       <c r="G129" t="inlineStr">
@@ -10153,7 +10153,7 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sluchac bez obrony</t>
+          <t xml:space="preserve">Slucham bez obrony</t>
         </is>
       </c>
       <c r="G130" t="inlineStr">
@@ -10231,7 +10231,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t xml:space="preserve">Relacje potrzebuja czasu</t>
+          <t xml:space="preserve">Daje relacjom czas</t>
         </is>
       </c>
       <c r="G131" t="inlineStr">
@@ -10309,7 +10309,7 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zaufanie rodzi sie powoli</t>
+          <t xml:space="preserve">Pozwalam, by zaufanie rodzilo sie powoli</t>
         </is>
       </c>
       <c r="G132" t="inlineStr">
@@ -10387,7 +10387,7 @@
       </c>
       <c r="F133" t="inlineStr">
         <is>
-          <t xml:space="preserve">Uczciwosc w rozmowie</t>
+          <t xml:space="preserve">Ucze sie uczciwosci w rozmowie</t>
         </is>
       </c>
       <c r="G133" t="inlineStr">
@@ -10465,7 +10465,7 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bliskosc bez manipulacji</t>
+          <t xml:space="preserve">Ucze sie bliskosci bez manipulacji</t>
         </is>
       </c>
       <c r="G134" t="inlineStr">
@@ -10543,7 +10543,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spotkanie zamiast walki</t>
+          <t xml:space="preserve">Wybieram spotkanie zamiast walki</t>
         </is>
       </c>
       <c r="G135" t="inlineStr">
@@ -10621,7 +10621,7 @@
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kiedy przestaje udowadniac racje</t>
+          <t xml:space="preserve">Przestaje udowadniac racje</t>
         </is>
       </c>
       <c r="G136" t="inlineStr">
@@ -10699,7 +10699,7 @@
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t xml:space="preserve">Byc obecnym</t>
+          <t xml:space="preserve">Ucze sie byc obecnym</t>
         </is>
       </c>
       <c r="G137" t="inlineStr">
@@ -10777,7 +10777,7 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t xml:space="preserve">Relacja jako przestrzen rozwoju</t>
+          <t xml:space="preserve">Traktuje relacje jak przestrzen rozwoju</t>
         </is>
       </c>
       <c r="G138" t="inlineStr">
@@ -10855,7 +10855,7 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t xml:space="preserve">Otworzyc sie na drugiego</t>
+          <t xml:space="preserve">Otwieram sie na drugiego</t>
         </is>
       </c>
       <c r="G139" t="inlineStr">
@@ -10933,7 +10933,7 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sluchac takze tego, co trudne</t>
+          <t xml:space="preserve">Slucham takze tego, co trudne</t>
         </is>
       </c>
       <c r="G140" t="inlineStr">
@@ -11011,7 +11011,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kiedy pojawia sie zrozumienie</t>
+          <t xml:space="preserve">Otwieram sie na zrozumienie</t>
         </is>
       </c>
       <c r="G141" t="inlineStr">
@@ -11089,7 +11089,7 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t xml:space="preserve">Budowanie zaufania</t>
+          <t xml:space="preserve">Buduje zaufanie</t>
         </is>
       </c>
       <c r="G142" t="inlineStr">
@@ -11167,7 +11167,7 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc w relacji</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc w relacji</t>
         </is>
       </c>
       <c r="G143" t="inlineStr">
@@ -11245,7 +11245,7 @@
       </c>
       <c r="F144" t="inlineStr">
         <is>
-          <t xml:space="preserve">Przyjecie drugiego czlowieka</t>
+          <t xml:space="preserve">Ucze sie przyjmowac drugiego czlowieka</t>
         </is>
       </c>
       <c r="G144" t="inlineStr">
@@ -11323,7 +11323,7 @@
       </c>
       <c r="F145" t="inlineStr">
         <is>
-          <t xml:space="preserve">Roznice miedzy nami</t>
+          <t xml:space="preserve">Przyjmuje roznice miedzy nami</t>
         </is>
       </c>
       <c r="G145" t="inlineStr">
@@ -11401,7 +11401,7 @@
       </c>
       <c r="F146" t="inlineStr">
         <is>
-          <t xml:space="preserve">Szacunek w rozmowie</t>
+          <t xml:space="preserve">Ucze sie szacunku w rozmowie</t>
         </is>
       </c>
       <c r="G146" t="inlineStr">
@@ -11479,7 +11479,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t xml:space="preserve">Miejsce na emocje w relacji</t>
+          <t xml:space="preserve">Robie miejsce na emocje w relacji</t>
         </is>
       </c>
       <c r="G147" t="inlineStr">
@@ -11557,7 +11557,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t xml:space="preserve">Relacje ucza cierpliwosci</t>
+          <t xml:space="preserve">Relacje ucza mnie cierpliwosci</t>
         </is>
       </c>
       <c r="G148" t="inlineStr">
@@ -11635,7 +11635,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t xml:space="preserve">Uczyc sie byc razem</t>
+          <t xml:space="preserve">Ucze sie byc razem</t>
         </is>
       </c>
       <c r="G149" t="inlineStr">
@@ -11713,7 +11713,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spotkanie bez masek</t>
+          <t xml:space="preserve">Spotykam bez masek</t>
         </is>
       </c>
       <c r="G150" t="inlineStr">
@@ -11791,7 +11791,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bliskosc i granice</t>
+          <t xml:space="preserve">Ucze sie bliskosci i granic</t>
         </is>
       </c>
       <c r="G151" t="inlineStr">
@@ -11869,7 +11869,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t xml:space="preserve">Relacje jako droga</t>
+          <t xml:space="preserve">Traktuje relacje jak droge</t>
         </is>
       </c>
       <c r="G152" t="inlineStr">
@@ -11947,7 +11947,7 @@
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t xml:space="preserve">Czlowiek potrzebuje czlowieka</t>
+          <t xml:space="preserve">Potrzebuje drugiego czlowieka</t>
         </is>
       </c>
       <c r="G153" t="inlineStr">
@@ -12025,7 +12025,7 @@
       </c>
       <c r="F154" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice zaczynaja sie od swiadomosci</t>
+          <t xml:space="preserve">Zaczynam od swiadomosci swoich granic</t>
         </is>
       </c>
       <c r="G154" t="inlineStr">
@@ -12103,7 +12103,7 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mowic "nie" bez poczucia winy</t>
+          <t xml:space="preserve">Mowie "nie" bez poczucia winy</t>
         </is>
       </c>
       <c r="G155" t="inlineStr">
@@ -12181,7 +12181,7 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice chronia relacje</t>
+          <t xml:space="preserve">Widze, ze granice chronia relacje</t>
         </is>
       </c>
       <c r="G156" t="inlineStr">
@@ -12259,7 +12259,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kiedy ucze sie siebie szanowac</t>
+          <t xml:space="preserve">Ucze sie siebie szanowac</t>
         </is>
       </c>
       <c r="G157" t="inlineStr">
@@ -12337,7 +12337,7 @@
       </c>
       <c r="F158" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odpowiedzialnosc za wlasne zycie</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za wlasne zycie</t>
         </is>
       </c>
       <c r="G158" t="inlineStr">
@@ -12415,7 +12415,7 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice to nie mur</t>
+          <t xml:space="preserve">Widze, ze granice to nie mur</t>
         </is>
       </c>
       <c r="G159" t="inlineStr">
@@ -12493,7 +12493,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice jako przestrzen wolnosci</t>
+          <t xml:space="preserve">Widze w granicach przestrzen wolnosci</t>
         </is>
       </c>
       <c r="G160" t="inlineStr">
@@ -12571,7 +12571,7 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t xml:space="preserve">Odrozniac pomoc od ratowania</t>
+          <t xml:space="preserve">Odrozniam pomoc od ratowania</t>
         </is>
       </c>
       <c r="G161" t="inlineStr">
@@ -12649,7 +12649,7 @@
       </c>
       <c r="F162" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zauwazyc wlasne potrzeby</t>
+          <t xml:space="preserve">Zauwazam wlasne potrzeby</t>
         </is>
       </c>
       <c r="G162" t="inlineStr">
@@ -12727,7 +12727,7 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice wobec przeszlosci</t>
+          <t xml:space="preserve">Stawiam granice wobec przeszlosci</t>
         </is>
       </c>
       <c r="G163" t="inlineStr">
@@ -12805,7 +12805,7 @@
       </c>
       <c r="F164" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice wobec manipulacji</t>
+          <t xml:space="preserve">Stawiam granice wobec manipulacji</t>
         </is>
       </c>
       <c r="G164" t="inlineStr">
@@ -12883,7 +12883,7 @@
       </c>
       <c r="F165" t="inlineStr">
         <is>
-          <t xml:space="preserve">Uczyc sie odmawiac</t>
+          <t xml:space="preserve">Ucze sie odmawiac</t>
         </is>
       </c>
       <c r="G165" t="inlineStr">
@@ -12961,7 +12961,7 @@
       </c>
       <c r="F166" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice wobec chaosu</t>
+          <t xml:space="preserve">Stawiam granice wobec chaosu</t>
         </is>
       </c>
       <c r="G166" t="inlineStr">
@@ -13039,7 +13039,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice wobec przemocy</t>
+          <t xml:space="preserve">Stawiam granice wobec przemocy</t>
         </is>
       </c>
       <c r="G167" t="inlineStr">
@@ -13117,7 +13117,7 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice wobec wlasnych impulsow</t>
+          <t xml:space="preserve">Stawiam granice wobec wlasnych impulsow</t>
         </is>
       </c>
       <c r="G168" t="inlineStr">
@@ -13195,7 +13195,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice wobec leku</t>
+          <t xml:space="preserve">Stawiam granice wobec leku</t>
         </is>
       </c>
       <c r="G169" t="inlineStr">
@@ -13273,7 +13273,7 @@
       </c>
       <c r="F170" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice wobec oczekiwan innych</t>
+          <t xml:space="preserve">Stawiam granice wobec oczekiwan innych</t>
         </is>
       </c>
       <c r="G170" t="inlineStr">
@@ -13351,7 +13351,7 @@
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice w relacjach rodzinnych</t>
+          <t xml:space="preserve">Stawiam granice w relacjach rodzinnych</t>
         </is>
       </c>
       <c r="G171" t="inlineStr">
@@ -13429,7 +13429,7 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice wobec pracy</t>
+          <t xml:space="preserve">Stawiam granice wobec pracy</t>
         </is>
       </c>
       <c r="G172" t="inlineStr">
@@ -13507,7 +13507,7 @@
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice wobec zmeczenia</t>
+          <t xml:space="preserve">Stawiam granice wobec zmeczenia</t>
         </is>
       </c>
       <c r="G173" t="inlineStr">
@@ -13585,7 +13585,7 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice jako akt odwagi</t>
+          <t xml:space="preserve">Stawiam granice jako akt odwagi</t>
         </is>
       </c>
       <c r="G174" t="inlineStr">
@@ -13663,7 +13663,7 @@
       </c>
       <c r="F175" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice wobec nalogu</t>
+          <t xml:space="preserve">Stawiam granice wobec nalogu</t>
         </is>
       </c>
       <c r="G175" t="inlineStr">
@@ -13741,7 +13741,7 @@
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice wobec destrukcji</t>
+          <t xml:space="preserve">Stawiam granice wobec destrukcji</t>
         </is>
       </c>
       <c r="G176" t="inlineStr">
@@ -13819,7 +13819,7 @@
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice wobec iluzji</t>
+          <t xml:space="preserve">Stawiam granice wobec iluzji</t>
         </is>
       </c>
       <c r="G177" t="inlineStr">
@@ -13897,7 +13897,7 @@
       </c>
       <c r="F178" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice wobec manipulacji emocjonalnej</t>
+          <t xml:space="preserve">Stawiam granice wobec manipulacji emocjonalnej</t>
         </is>
       </c>
       <c r="G178" t="inlineStr">
@@ -13975,7 +13975,7 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice wobec chaosu w glowie</t>
+          <t xml:space="preserve">Stawiam granice wobec chaosu w glowie</t>
         </is>
       </c>
       <c r="G179" t="inlineStr">
@@ -14053,7 +14053,7 @@
       </c>
       <c r="F180" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice jako troska o siebie</t>
+          <t xml:space="preserve">Traktuje granice jak troske o siebie</t>
         </is>
       </c>
       <c r="G180" t="inlineStr">
@@ -14131,7 +14131,7 @@
       </c>
       <c r="F181" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice jako wyraz szacunku</t>
+          <t xml:space="preserve">Traktuje granice jak wyraz szacunku</t>
         </is>
       </c>
       <c r="G181" t="inlineStr">
@@ -14209,7 +14209,7 @@
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice jako warunek zdrowia</t>
+          <t xml:space="preserve">Traktuje granice jak warunek zdrowia</t>
         </is>
       </c>
       <c r="G182" t="inlineStr">
@@ -14287,7 +14287,7 @@
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t xml:space="preserve">Granice buduja bezpieczenstwo</t>
+          <t xml:space="preserve">Widze, jak granice buduja bezpieczenstwo</t>
         </is>
       </c>
       <c r="G183" t="inlineStr">
@@ -14365,7 +14365,7 @@
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t xml:space="preserve">Czlowiek zdrowieje miedzy ludzmi</t>
+          <t xml:space="preserve">Zdrowieje miedzy ludzmi</t>
         </is>
       </c>
       <c r="G184" t="inlineStr">
@@ -14443,7 +14443,7 @@
       </c>
       <c r="F185" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sila wspolnoty</t>
+          <t xml:space="preserve">Czerpie sile ze wspolnoty</t>
         </is>
       </c>
       <c r="G185" t="inlineStr">
@@ -14521,7 +14521,7 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wspolnota jako lustro</t>
+          <t xml:space="preserve">Wspolnota staje sie dla mnie lustrem</t>
         </is>
       </c>
       <c r="G186" t="inlineStr">
@@ -14599,7 +14599,7 @@
       </c>
       <c r="F187" t="inlineStr">
         <is>
-          <t xml:space="preserve">Spotkanie w prawdzie</t>
+          <t xml:space="preserve">Spotykam sie w prawdzie</t>
         </is>
       </c>
       <c r="G187" t="inlineStr">
@@ -14677,7 +14677,7 @@
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wspolnota bez masek</t>
+          <t xml:space="preserve">Ucze sie wspolnoty bez masek</t>
         </is>
       </c>
       <c r="G188" t="inlineStr">
@@ -14755,7 +14755,7 @@
       </c>
       <c r="F189" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielenie sie doswiadczeniem</t>
+          <t xml:space="preserve">Dziele sie doswiadczeniem</t>
         </is>
       </c>
       <c r="G189" t="inlineStr">
@@ -14833,7 +14833,7 @@
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sluchanie historii innych</t>
+          <t xml:space="preserve">Slucham historii innych</t>
         </is>
       </c>
       <c r="G190" t="inlineStr">
@@ -14911,7 +14911,7 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wspolnota daje nadzieje</t>
+          <t xml:space="preserve">Wspolnota daje mi nadzieje</t>
         </is>
       </c>
       <c r="G191" t="inlineStr">
@@ -14989,7 +14989,7 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wspolnota jako przestrzen zmiany</t>
+          <t xml:space="preserve">Wspolnota staje sie dla mnie przestrzenia zmiany</t>
         </is>
       </c>
       <c r="G192" t="inlineStr">
@@ -15067,7 +15067,7 @@
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t xml:space="preserve">Uczyc sie byc razem</t>
+          <t xml:space="preserve">Ucze sie byc razem</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
@@ -15145,7 +15145,7 @@
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wspolnota bez oceniania</t>
+          <t xml:space="preserve">Ucze sie wspolnoty bez oceniania</t>
         </is>
       </c>
       <c r="G194" t="inlineStr">
@@ -15223,7 +15223,7 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wspolnota jako wsparcie</t>
+          <t xml:space="preserve">Wspolnota staje sie dla mnie wsparciem</t>
         </is>
       </c>
       <c r="G195" t="inlineStr">
@@ -15301,7 +15301,7 @@
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kazdy wnosi swoja historie</t>
+          <t xml:space="preserve">Wnosze swoja historie</t>
         </is>
       </c>
       <c r="G196" t="inlineStr">
@@ -15379,7 +15379,7 @@
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wspolnota jako szkola relacji</t>
+          <t xml:space="preserve">Wspolnota staje sie dla mnie szkola relacji</t>
         </is>
       </c>
       <c r="G197" t="inlineStr">
@@ -15457,7 +15457,7 @@
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wspolnota i odpowiedzialnosc</t>
+          <t xml:space="preserve">Ucze sie wspolnoty i odpowiedzialnosci</t>
         </is>
       </c>
       <c r="G198" t="inlineStr">
@@ -15535,7 +15535,7 @@
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wspolnota jako droga</t>
+          <t xml:space="preserve">Wspolnota staje sie dla mnie droga</t>
         </is>
       </c>
       <c r="G199" t="inlineStr">
@@ -15613,7 +15613,7 @@
       </c>
       <c r="F200" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sila bycia razem</t>
+          <t xml:space="preserve">Odkrywam sile bycia razem</t>
         </is>
       </c>
       <c r="G200" t="inlineStr">
@@ -15691,7 +15691,7 @@
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wspolnota i zaufanie</t>
+          <t xml:space="preserve">Ucze sie wspolnoty i zaufania</t>
         </is>
       </c>
       <c r="G201" t="inlineStr">
@@ -15769,7 +15769,7 @@
       </c>
       <c r="F202" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wspolnota i szczerosc</t>
+          <t xml:space="preserve">Ucze sie wspolnoty i szczerosci</t>
         </is>
       </c>
       <c r="G202" t="inlineStr">
@@ -15847,7 +15847,7 @@
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wspolnota i odwaga</t>
+          <t xml:space="preserve">Ucze sie wspolnoty i odwagi</t>
         </is>
       </c>
       <c r="G203" t="inlineStr">
@@ -15925,7 +15925,7 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wspolnota i pokora</t>
+          <t xml:space="preserve">Ucze sie wspolnoty i pokory</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
@@ -16003,7 +16003,7 @@
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wspolnota jako miejsce zdrowienia</t>
+          <t xml:space="preserve">Wspolnota staje sie dla mnie miejscem zdrowienia</t>
         </is>
       </c>
       <c r="G205" t="inlineStr">
@@ -16081,7 +16081,7 @@
       </c>
       <c r="F206" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wspolnota daje perspektywe</t>
+          <t xml:space="preserve">Wspolnota daje mi perspektywe</t>
         </is>
       </c>
       <c r="G206" t="inlineStr">
@@ -16159,7 +16159,7 @@
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wspolnota i nadzieja</t>
+          <t xml:space="preserve">Widze nadzieje we wspolnocie</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
@@ -16237,7 +16237,7 @@
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wspolnota jako dom</t>
+          <t xml:space="preserve">Wspolnota staje sie dla mnie domem</t>
         </is>
       </c>
       <c r="G208" t="inlineStr">
@@ -16315,7 +16315,7 @@
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wspolnota i codziennosc</t>
+          <t xml:space="preserve">Ucze sie wspolnoty w codziennosci</t>
         </is>
       </c>
       <c r="G209" t="inlineStr">
@@ -16393,7 +16393,7 @@
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wspolnota i rozmowa</t>
+          <t xml:space="preserve">Ucze sie wspolnoty w rozmowie</t>
         </is>
       </c>
       <c r="G210" t="inlineStr">
@@ -16471,7 +16471,7 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wspolnota i obecnosc</t>
+          <t xml:space="preserve">Ucze sie wspolnoty w obecnosci</t>
         </is>
       </c>
       <c r="G211" t="inlineStr">
@@ -16549,7 +16549,7 @@
       </c>
       <c r="F212" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wspolnota i wzrost</t>
+          <t xml:space="preserve">Ucze sie wspolnoty we wzroscie</t>
         </is>
       </c>
       <c r="G212" t="inlineStr">
@@ -16627,7 +16627,7 @@
       </c>
       <c r="F213" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wspolnota i odpowiedzialnosc</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc we wspolnocie</t>
         </is>
       </c>
       <c r="G213" t="inlineStr">
@@ -16705,7 +16705,7 @@
       </c>
       <c r="F214" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wspolnota jako droga powrotu</t>
+          <t xml:space="preserve">Wspolnota staje sie moja droga powrotu</t>
         </is>
       </c>
       <c r="G214" t="inlineStr">
@@ -16783,7 +16783,7 @@
       </c>
       <c r="F215" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora zaczyna sie od prawdy</t>
+          <t xml:space="preserve">Ucze sie pokory zaczynajac od prawdy</t>
         </is>
       </c>
       <c r="G215" t="inlineStr">
@@ -16861,7 +16861,7 @@
       </c>
       <c r="F216" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec zycia</t>
+          <t xml:space="preserve">Ucze sie pokory wobec zycia</t>
         </is>
       </c>
       <c r="G216" t="inlineStr">
@@ -16939,7 +16939,7 @@
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec wlasnych bledow</t>
+          <t xml:space="preserve">Ucze sie pokory wobec wlasnych bledow</t>
         </is>
       </c>
       <c r="G217" t="inlineStr">
@@ -17017,7 +17017,7 @@
       </c>
       <c r="F218" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec innych ludzi</t>
+          <t xml:space="preserve">Ucze sie pokory wobec innych ludzi</t>
         </is>
       </c>
       <c r="G218" t="inlineStr">
@@ -17095,7 +17095,7 @@
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec procesu</t>
+          <t xml:space="preserve">Ucze sie pokory wobec procesu</t>
         </is>
       </c>
       <c r="G219" t="inlineStr">
@@ -17173,7 +17173,7 @@
       </c>
       <c r="F220" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec emocji</t>
+          <t xml:space="preserve">Ucze sie pokory wobec emocji</t>
         </is>
       </c>
       <c r="G220" t="inlineStr">
@@ -17251,7 +17251,7 @@
       </c>
       <c r="F221" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec zmiany</t>
+          <t xml:space="preserve">Ucze sie pokory wobec zmiany</t>
         </is>
       </c>
       <c r="G221" t="inlineStr">
@@ -17329,7 +17329,7 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec czasu</t>
+          <t xml:space="preserve">Ucze sie pokory wobec czasu</t>
         </is>
       </c>
       <c r="G222" t="inlineStr">
@@ -17407,7 +17407,7 @@
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec doswiadczenia</t>
+          <t xml:space="preserve">Ucze sie pokory wobec doswiadczenia</t>
         </is>
       </c>
       <c r="G223" t="inlineStr">
@@ -17485,7 +17485,7 @@
       </c>
       <c r="F224" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec wiedzy</t>
+          <t xml:space="preserve">Ucze sie pokory wobec wiedzy</t>
         </is>
       </c>
       <c r="G224" t="inlineStr">
@@ -17563,7 +17563,7 @@
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec wlasnych ograniczen</t>
+          <t xml:space="preserve">Ucze sie pokory wobec wlasnych ograniczen</t>
         </is>
       </c>
       <c r="G225" t="inlineStr">
@@ -17641,7 +17641,7 @@
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec relacji</t>
+          <t xml:space="preserve">Ucze sie pokory wobec relacji</t>
         </is>
       </c>
       <c r="G226" t="inlineStr">
@@ -17719,7 +17719,7 @@
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec przeszlosci</t>
+          <t xml:space="preserve">Ucze sie pokory wobec przeszlosci</t>
         </is>
       </c>
       <c r="G227" t="inlineStr">
@@ -17797,7 +17797,7 @@
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec terazniejszosci</t>
+          <t xml:space="preserve">Ucze sie pokory wobec terazniejszosci</t>
         </is>
       </c>
       <c r="G228" t="inlineStr">
@@ -17875,7 +17875,7 @@
       </c>
       <c r="F229" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec przyszlosci</t>
+          <t xml:space="preserve">Ucze sie pokory wobec przyszlosci</t>
         </is>
       </c>
       <c r="G229" t="inlineStr">
@@ -17953,7 +17953,7 @@
       </c>
       <c r="F230" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora jako sila</t>
+          <t xml:space="preserve">Odkrywam, ze pokora jest sila</t>
         </is>
       </c>
       <c r="G230" t="inlineStr">
@@ -18031,7 +18031,7 @@
       </c>
       <c r="F231" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora jako uczciwosc</t>
+          <t xml:space="preserve">Odkrywam, ze pokora jest uczciwoscia</t>
         </is>
       </c>
       <c r="G231" t="inlineStr">
@@ -18109,7 +18109,7 @@
       </c>
       <c r="F232" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora jako odwaga</t>
+          <t xml:space="preserve">Odkrywam, ze pokora jest odwaga</t>
         </is>
       </c>
       <c r="G232" t="inlineStr">
@@ -18187,7 +18187,7 @@
       </c>
       <c r="F233" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec prawdy</t>
+          <t xml:space="preserve">Ucze sie pokory wobec prawdy</t>
         </is>
       </c>
       <c r="G233" t="inlineStr">
@@ -18265,7 +18265,7 @@
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec zycia codziennego</t>
+          <t xml:space="preserve">Ucze sie pokory wobec zycia codziennego</t>
         </is>
       </c>
       <c r="G234" t="inlineStr">
@@ -18343,7 +18343,7 @@
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec pracy nad soba</t>
+          <t xml:space="preserve">Ucze sie pokory wobec pracy nad soba</t>
         </is>
       </c>
       <c r="G235" t="inlineStr">
@@ -18421,7 +18421,7 @@
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec wspolnoty</t>
+          <t xml:space="preserve">Ucze sie pokory wobec wspolnoty</t>
         </is>
       </c>
       <c r="G236" t="inlineStr">
@@ -18499,7 +18499,7 @@
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec slabosci</t>
+          <t xml:space="preserve">Ucze sie pokory wobec slabosci</t>
         </is>
       </c>
       <c r="G237" t="inlineStr">
@@ -18577,7 +18577,7 @@
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec cierpienia</t>
+          <t xml:space="preserve">Ucze sie pokory wobec cierpienia</t>
         </is>
       </c>
       <c r="G238" t="inlineStr">
@@ -18655,7 +18655,7 @@
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec radosci</t>
+          <t xml:space="preserve">Ucze sie pokory wobec radosci</t>
         </is>
       </c>
       <c r="G239" t="inlineStr">
@@ -18733,7 +18733,7 @@
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec zmeczenia</t>
+          <t xml:space="preserve">Ucze sie pokory wobec zmeczenia</t>
         </is>
       </c>
       <c r="G240" t="inlineStr">
@@ -18811,7 +18811,7 @@
       </c>
       <c r="F241" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec nadziei</t>
+          <t xml:space="preserve">Ucze sie pokory wobec nadziei</t>
         </is>
       </c>
       <c r="G241" t="inlineStr">
@@ -18889,7 +18889,7 @@
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec milosci</t>
+          <t xml:space="preserve">Ucze sie pokory wobec milosci</t>
         </is>
       </c>
       <c r="G242" t="inlineStr">
@@ -18967,7 +18967,7 @@
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec drogi</t>
+          <t xml:space="preserve">Ucze sie pokory wobec drogi</t>
         </is>
       </c>
       <c r="G243" t="inlineStr">
@@ -19045,7 +19045,7 @@
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora wobec sensu</t>
+          <t xml:space="preserve">Ucze sie pokory wobec sensu</t>
         </is>
       </c>
       <c r="G244" t="inlineStr">
@@ -19123,7 +19123,7 @@
       </c>
       <c r="F245" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pokora jako wolnosc</t>
+          <t xml:space="preserve">Odkrywam, ze pokora jest wolnoscia</t>
         </is>
       </c>
       <c r="G245" t="inlineStr">
@@ -19201,7 +19201,7 @@
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zmiana zaczyna sie w srodku</t>
+          <t xml:space="preserve">Zmiana zaczyna sie we mnie</t>
         </is>
       </c>
       <c r="G246" t="inlineStr">
@@ -19279,7 +19279,7 @@
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zmiana wymaga odwagi</t>
+          <t xml:space="preserve">Wchodze w zmiane z odwaga</t>
         </is>
       </c>
       <c r="G247" t="inlineStr">
@@ -19357,7 +19357,7 @@
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zmiana zaczyna sie od decyzji</t>
+          <t xml:space="preserve">Zmiane zaczynam od decyzji</t>
         </is>
       </c>
       <c r="G248" t="inlineStr">
@@ -19435,7 +19435,7 @@
       </c>
       <c r="F249" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zmiana potrzebuje czasu</t>
+          <t xml:space="preserve">Daje zmianie czas</t>
         </is>
       </c>
       <c r="G249" t="inlineStr">
@@ -19513,7 +19513,7 @@
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zmiana nie jest linia prosta</t>
+          <t xml:space="preserve">Widze, ze zmiana nie jest linia prosta</t>
         </is>
       </c>
       <c r="G250" t="inlineStr">
@@ -19591,7 +19591,7 @@
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jeden dzien tez jest zmiana</t>
+          <t xml:space="preserve">Jeden moj dzien tez jest zmiana</t>
         </is>
       </c>
       <c r="G251" t="inlineStr">
@@ -19669,7 +19669,7 @@
       </c>
       <c r="F252" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zmiana jako droga</t>
+          <t xml:space="preserve">Traktuje zmiane jak droge</t>
         </is>
       </c>
       <c r="G252" t="inlineStr">
@@ -19747,7 +19747,7 @@
       </c>
       <c r="F253" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zmiana zaczyna sie od powrotu</t>
+          <t xml:space="preserve">Zmiane zaczynam od powrotu</t>
         </is>
       </c>
       <c r="G253" t="inlineStr">
@@ -19825,7 +19825,7 @@
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nawyk buduje przyszlosc</t>
+          <t xml:space="preserve">Widze, jak nawyk buduje moja przyszlosc</t>
         </is>
       </c>
       <c r="G254" t="inlineStr">
@@ -19903,7 +19903,7 @@
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t xml:space="preserve">Male kroki tez maja znaczenie</t>
+          <t xml:space="preserve">Wierze, ze male kroki tez maja znaczenie</t>
         </is>
       </c>
       <c r="G255" t="inlineStr">
@@ -19981,7 +19981,7 @@
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zmiana i lek przed nawrotem</t>
+          <t xml:space="preserve">Widze zmiane i lek przed nawrotem</t>
         </is>
       </c>
       <c r="G256" t="inlineStr">
@@ -20059,7 +20059,7 @@
       </c>
       <c r="F257" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzien po potknieciu</t>
+          <t xml:space="preserve">Wracam po potknieciu</t>
         </is>
       </c>
       <c r="G257" t="inlineStr">
@@ -20137,7 +20137,7 @@
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nie przekreslac wszystkiego</t>
+          <t xml:space="preserve">Nie przekreslam wszystkiego</t>
         </is>
       </c>
       <c r="G258" t="inlineStr">
@@ -20215,7 +20215,7 @@
       </c>
       <c r="F259" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wracac do rytmu</t>
+          <t xml:space="preserve">Wracam do rytmu</t>
         </is>
       </c>
       <c r="G259" t="inlineStr">
@@ -20293,7 +20293,7 @@
       </c>
       <c r="F260" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cialo tez potrzebuje zmiany</t>
+          <t xml:space="preserve">Widze, ze moje cialo tez potrzebuje zmiany</t>
         </is>
       </c>
       <c r="G260" t="inlineStr">
@@ -20371,7 +20371,7 @@
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sen, jedzenie i spokoj</t>
+          <t xml:space="preserve">Dbam o sen, jedzenie i spokoj</t>
         </is>
       </c>
       <c r="G261" t="inlineStr">
@@ -20449,7 +20449,7 @@
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wieczor bywa trudny</t>
+          <t xml:space="preserve">Widze, ze wieczor bywa trudny</t>
         </is>
       </c>
       <c r="G262" t="inlineStr">
@@ -20527,7 +20527,7 @@
       </c>
       <c r="F263" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zmiana potrzebuje planu</t>
+          <t xml:space="preserve">Daje zmianie plan</t>
         </is>
       </c>
       <c r="G263" t="inlineStr">
@@ -20605,7 +20605,7 @@
       </c>
       <c r="F264" t="inlineStr">
         <is>
-          <t xml:space="preserve">Prosic o pomoc wczesniej</t>
+          <t xml:space="preserve">Prosze o pomoc wczesniej</t>
         </is>
       </c>
       <c r="G264" t="inlineStr">
@@ -20683,7 +20683,7 @@
       </c>
       <c r="F265" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zmiana i cierpliwosc</t>
+          <t xml:space="preserve">Daje zmianie cierpliwosc</t>
         </is>
       </c>
       <c r="G265" t="inlineStr">
@@ -20761,7 +20761,7 @@
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zmiana jako praktyka</t>
+          <t xml:space="preserve">Traktuje zmiane jak praktyke</t>
         </is>
       </c>
       <c r="G266" t="inlineStr">
@@ -20839,7 +20839,7 @@
       </c>
       <c r="F267" t="inlineStr">
         <is>
-          <t xml:space="preserve">Powtarzac to, co dziala</t>
+          <t xml:space="preserve">Powtarzam to, co dziala</t>
         </is>
       </c>
       <c r="G267" t="inlineStr">
@@ -20917,7 +20917,7 @@
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zmiana w relacjach</t>
+          <t xml:space="preserve">Widze zmiane w relacjach</t>
         </is>
       </c>
       <c r="G268" t="inlineStr">
@@ -20995,7 +20995,7 @@
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nie wracac do starych wymowek</t>
+          <t xml:space="preserve">Nie wracam do starych wymowek</t>
         </is>
       </c>
       <c r="G269" t="inlineStr">
@@ -21073,7 +21073,7 @@
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zmiana i odpowiedzialnosc</t>
+          <t xml:space="preserve">Biore odpowiedzialnosc za zmiane</t>
         </is>
       </c>
       <c r="G270" t="inlineStr">
@@ -21151,7 +21151,7 @@
       </c>
       <c r="F271" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zmiana i codzienna rutyna</t>
+          <t xml:space="preserve">Ukladam zmiane w codziennej rutynie</t>
         </is>
       </c>
       <c r="G271" t="inlineStr">
@@ -21229,7 +21229,7 @@
       </c>
       <c r="F272" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zmiana jako wybor na dzis</t>
+          <t xml:space="preserve">Wybieram zmiane na dzis</t>
         </is>
       </c>
       <c r="G272" t="inlineStr">
@@ -21307,7 +21307,7 @@
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zmiana jako wytrwalosc</t>
+          <t xml:space="preserve">Trwam w zmianie</t>
         </is>
       </c>
       <c r="G273" t="inlineStr">
@@ -21385,7 +21385,7 @@
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zmiana jako nadzieja</t>
+          <t xml:space="preserve">Widze w zmianie nadzieje</t>
         </is>
       </c>
       <c r="G274" t="inlineStr">
@@ -21463,7 +21463,7 @@
       </c>
       <c r="F275" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zmiana jako nowe zycie</t>
+          <t xml:space="preserve">Wchodze w nowe zycie</t>
         </is>
       </c>
       <c r="G275" t="inlineStr">
@@ -21541,7 +21541,7 @@
       </c>
       <c r="F276" t="inlineStr">
         <is>
-          <t xml:space="preserve">Po co sie dzis zatrzymac</t>
+          <t xml:space="preserve">Szukam sensu tego zatrzymania</t>
         </is>
       </c>
       <c r="G276" t="inlineStr">
@@ -21619,7 +21619,7 @@
       </c>
       <c r="F277" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens jednego uczciwego dnia</t>
+          <t xml:space="preserve">Widze sens jednego uczciwego dnia</t>
         </is>
       </c>
       <c r="G277" t="inlineStr">
@@ -21697,7 +21697,7 @@
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens malego kroku</t>
+          <t xml:space="preserve">Widze sens malego kroku</t>
         </is>
       </c>
       <c r="G278" t="inlineStr">
@@ -21775,7 +21775,7 @@
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens trzymania granic</t>
+          <t xml:space="preserve">Widze sens trzymania granic</t>
         </is>
       </c>
       <c r="G279" t="inlineStr">
@@ -21853,7 +21853,7 @@
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens proszenia o pomoc</t>
+          <t xml:space="preserve">Widze sens proszenia o pomoc</t>
         </is>
       </c>
       <c r="G280" t="inlineStr">
@@ -21931,7 +21931,7 @@
       </c>
       <c r="F281" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens planu dnia</t>
+          <t xml:space="preserve">Widze sens planu dnia</t>
         </is>
       </c>
       <c r="G281" t="inlineStr">
@@ -22009,7 +22009,7 @@
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens nazywania uczuc</t>
+          <t xml:space="preserve">Widze sens nazywania uczuc</t>
         </is>
       </c>
       <c r="G282" t="inlineStr">
@@ -22087,7 +22087,7 @@
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens powiedzenia prawdy</t>
+          <t xml:space="preserve">Widze sens powiedzenia prawdy</t>
         </is>
       </c>
       <c r="G283" t="inlineStr">
@@ -22165,7 +22165,7 @@
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens zwyklej obecnosci</t>
+          <t xml:space="preserve">Widze sens zwyklej obecnosci</t>
         </is>
       </c>
       <c r="G284" t="inlineStr">
@@ -22243,7 +22243,7 @@
       </c>
       <c r="F285" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens wyjscia z samotnosci</t>
+          <t xml:space="preserve">Widze sens wyjscia z samotnosci</t>
         </is>
       </c>
       <c r="G285" t="inlineStr">
@@ -22321,7 +22321,7 @@
       </c>
       <c r="F286" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens rozmowy zamiast ucieczki</t>
+          <t xml:space="preserve">Widze sens rozmowy zamiast ucieczki</t>
         </is>
       </c>
       <c r="G286" t="inlineStr">
@@ -22399,7 +22399,7 @@
       </c>
       <c r="F287" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens odpoczynku</t>
+          <t xml:space="preserve">Widze sens odpoczynku</t>
         </is>
       </c>
       <c r="G287" t="inlineStr">
@@ -22477,7 +22477,7 @@
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens dbania o cialo</t>
+          <t xml:space="preserve">Widze sens dbania o cialo</t>
         </is>
       </c>
       <c r="G288" t="inlineStr">
@@ -22555,7 +22555,7 @@
       </c>
       <c r="F289" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens wytrwania w kryzysie</t>
+          <t xml:space="preserve">Widze sens wytrwania w kryzysie</t>
         </is>
       </c>
       <c r="G289" t="inlineStr">
@@ -22633,7 +22633,7 @@
       </c>
       <c r="F290" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens zaczynania od nowa</t>
+          <t xml:space="preserve">Widze sens zaczynania od nowa</t>
         </is>
       </c>
       <c r="G290" t="inlineStr">
@@ -22711,7 +22711,7 @@
       </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens przyjecia wlasnej historii</t>
+          <t xml:space="preserve">Widze sens przyjecia wlasnej historii</t>
         </is>
       </c>
       <c r="G291" t="inlineStr">
@@ -22789,7 +22789,7 @@
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens naprawiania szkod</t>
+          <t xml:space="preserve">Widze sens naprawiania szkod</t>
         </is>
       </c>
       <c r="G292" t="inlineStr">
@@ -22867,7 +22867,7 @@
       </c>
       <c r="F293" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens codziennych decyzji</t>
+          <t xml:space="preserve">Widze sens codziennych decyzji</t>
         </is>
       </c>
       <c r="G293" t="inlineStr">
@@ -22945,7 +22945,7 @@
       </c>
       <c r="F294" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens wspolnoty</t>
+          <t xml:space="preserve">Widze sens wspolnoty</t>
         </is>
       </c>
       <c r="G294" t="inlineStr">
@@ -23023,7 +23023,7 @@
       </c>
       <c r="F295" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens cierpliwosci</t>
+          <t xml:space="preserve">Widze sens cierpliwosci</t>
         </is>
       </c>
       <c r="G295" t="inlineStr">
@@ -23101,7 +23101,7 @@
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens pokory</t>
+          <t xml:space="preserve">Widze sens pokory</t>
         </is>
       </c>
       <c r="G296" t="inlineStr">
@@ -23179,7 +23179,7 @@
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens wytrwalosci</t>
+          <t xml:space="preserve">Widze sens wytrwalosci</t>
         </is>
       </c>
       <c r="G297" t="inlineStr">
@@ -23257,7 +23257,7 @@
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens pracy nad soba</t>
+          <t xml:space="preserve">Widze sens pracy nad soba</t>
         </is>
       </c>
       <c r="G298" t="inlineStr">
@@ -23335,7 +23335,7 @@
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens przebaczenia</t>
+          <t xml:space="preserve">Widze sens przebaczenia</t>
         </is>
       </c>
       <c r="G299" t="inlineStr">
@@ -23413,7 +23413,7 @@
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens przyjmowania dobra</t>
+          <t xml:space="preserve">Widze sens przyjmowania dobra</t>
         </is>
       </c>
       <c r="G300" t="inlineStr">
@@ -23491,7 +23491,7 @@
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens wdziecznosci</t>
+          <t xml:space="preserve">Widze sens wdziecznosci</t>
         </is>
       </c>
       <c r="G301" t="inlineStr">
@@ -23569,7 +23569,7 @@
       </c>
       <c r="F302" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens dawania innym</t>
+          <t xml:space="preserve">Widze sens dawania innym</t>
         </is>
       </c>
       <c r="G302" t="inlineStr">
@@ -23647,7 +23647,7 @@
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens zwyczajnosci</t>
+          <t xml:space="preserve">Widze sens zwyczajnosci</t>
         </is>
       </c>
       <c r="G303" t="inlineStr">
@@ -23725,7 +23725,7 @@
       </c>
       <c r="F304" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens nadziei</t>
+          <t xml:space="preserve">Widze sens nadziei</t>
         </is>
       </c>
       <c r="G304" t="inlineStr">
@@ -23803,7 +23803,7 @@
       </c>
       <c r="F305" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens dalszej drogi</t>
+          <t xml:space="preserve">Widze sens dalszej drogi</t>
         </is>
       </c>
       <c r="G305" t="inlineStr">
@@ -23881,7 +23881,7 @@
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sens bycia tu dzisiaj</t>
+          <t xml:space="preserve">Widze sens bycia tu dzisiaj</t>
         </is>
       </c>
       <c r="G306" t="inlineStr">
@@ -23959,7 +23959,7 @@
       </c>
       <c r="F307" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za to, ze zyje</t>
+          <t xml:space="preserve">Jestem wdzieczny za to, ze zyje</t>
         </is>
       </c>
       <c r="G307" t="inlineStr">
@@ -24037,7 +24037,7 @@
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za dzien bez ucieczki</t>
+          <t xml:space="preserve">Jestem wdzieczny za dzien bez ucieczki</t>
         </is>
       </c>
       <c r="G308" t="inlineStr">
@@ -24115,7 +24115,7 @@
       </c>
       <c r="F309" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za ludzi obok</t>
+          <t xml:space="preserve">Jestem wdzieczny za ludzi obok</t>
         </is>
       </c>
       <c r="G309" t="inlineStr">
@@ -24193,7 +24193,7 @@
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za telefon, ktory wykonalem</t>
+          <t xml:space="preserve">Jestem wdzieczny za telefon, ktory wykonalem</t>
         </is>
       </c>
       <c r="G310" t="inlineStr">
@@ -24271,7 +24271,7 @@
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za pomoc, ktora przyjalem</t>
+          <t xml:space="preserve">Jestem wdzieczny za pomoc, ktora przyjalem</t>
         </is>
       </c>
       <c r="G311" t="inlineStr">
@@ -24349,7 +24349,7 @@
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za zwykly spokoj</t>
+          <t xml:space="preserve">Jestem wdzieczny za zwykly spokoj</t>
         </is>
       </c>
       <c r="G312" t="inlineStr">
@@ -24427,7 +24427,7 @@
       </c>
       <c r="F313" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za cialo, ktore niesie</t>
+          <t xml:space="preserve">Jestem wdzieczny za cialo, ktore mnie niesie</t>
         </is>
       </c>
       <c r="G313" t="inlineStr">
@@ -24505,7 +24505,7 @@
       </c>
       <c r="F314" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za sen</t>
+          <t xml:space="preserve">Jestem wdzieczny za sen</t>
         </is>
       </c>
       <c r="G314" t="inlineStr">
@@ -24583,7 +24583,7 @@
       </c>
       <c r="F315" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za posilek</t>
+          <t xml:space="preserve">Jestem wdzieczny za posilek</t>
         </is>
       </c>
       <c r="G315" t="inlineStr">
@@ -24661,7 +24661,7 @@
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za dom</t>
+          <t xml:space="preserve">Jestem wdzieczny za dom</t>
         </is>
       </c>
       <c r="G316" t="inlineStr">
@@ -24739,7 +24739,7 @@
       </c>
       <c r="F317" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za rozmowe</t>
+          <t xml:space="preserve">Jestem wdzieczny za rozmowe</t>
         </is>
       </c>
       <c r="G317" t="inlineStr">
@@ -24817,7 +24817,7 @@
       </c>
       <c r="F318" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za obecnosc</t>
+          <t xml:space="preserve">Jestem wdzieczny za obecnosc</t>
         </is>
       </c>
       <c r="G318" t="inlineStr">
@@ -24895,7 +24895,7 @@
       </c>
       <c r="F319" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za plan na dzis</t>
+          <t xml:space="preserve">Jestem wdzieczny za plan na dzis</t>
         </is>
       </c>
       <c r="G319" t="inlineStr">
@@ -24973,7 +24973,7 @@
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za granice</t>
+          <t xml:space="preserve">Jestem wdzieczny za granice</t>
         </is>
       </c>
       <c r="G320" t="inlineStr">
@@ -25051,7 +25051,7 @@
       </c>
       <c r="F321" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za odwage powiedzenia prawdy</t>
+          <t xml:space="preserve">Jestem wdzieczny za odwage powiedzenia prawdy</t>
         </is>
       </c>
       <c r="G321" t="inlineStr">
@@ -25129,7 +25129,7 @@
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za zatrzymanie</t>
+          <t xml:space="preserve">Jestem wdzieczny za zatrzymanie</t>
         </is>
       </c>
       <c r="G322" t="inlineStr">
@@ -25207,7 +25207,7 @@
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za cierpliwosc</t>
+          <t xml:space="preserve">Jestem wdzieczny za cierpliwosc</t>
         </is>
       </c>
       <c r="G323" t="inlineStr">
@@ -25285,7 +25285,7 @@
       </c>
       <c r="F324" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za ludzi, ktorzy nie odpuscili</t>
+          <t xml:space="preserve">Jestem wdzieczny za ludzi, ktorzy nie odpuscili</t>
         </is>
       </c>
       <c r="G324" t="inlineStr">
@@ -25363,7 +25363,7 @@
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za wspolnote</t>
+          <t xml:space="preserve">Jestem wdzieczny za wspolnote</t>
         </is>
       </c>
       <c r="G325" t="inlineStr">
@@ -25441,7 +25441,7 @@
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za male zwyciestwa</t>
+          <t xml:space="preserve">Jestem wdzieczny za male zwyciestwa</t>
         </is>
       </c>
       <c r="G326" t="inlineStr">
@@ -25519,7 +25519,7 @@
       </c>
       <c r="F327" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za dzien dzisiejszy</t>
+          <t xml:space="preserve">Jestem wdzieczny za dzien dzisiejszy</t>
         </is>
       </c>
       <c r="G327" t="inlineStr">
@@ -25597,7 +25597,7 @@
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za nauke z potkniec</t>
+          <t xml:space="preserve">Jestem wdzieczny za nauke z potkniec</t>
         </is>
       </c>
       <c r="G328" t="inlineStr">
@@ -25675,7 +25675,7 @@
       </c>
       <c r="F329" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za zmiane, ktora rosnie powoli</t>
+          <t xml:space="preserve">Jestem wdzieczny za zmiane, ktora rosnie powoli</t>
         </is>
       </c>
       <c r="G329" t="inlineStr">
@@ -25753,7 +25753,7 @@
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za nadzieje</t>
+          <t xml:space="preserve">Jestem wdzieczny za nadzieje</t>
         </is>
       </c>
       <c r="G330" t="inlineStr">
@@ -25831,7 +25831,7 @@
       </c>
       <c r="F331" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za sens</t>
+          <t xml:space="preserve">Jestem wdzieczny za sens</t>
         </is>
       </c>
       <c r="G331" t="inlineStr">
@@ -25909,7 +25909,7 @@
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za mozliwosc naprawy</t>
+          <t xml:space="preserve">Jestem wdzieczny za mozliwosc naprawy</t>
         </is>
       </c>
       <c r="G332" t="inlineStr">
@@ -25987,7 +25987,7 @@
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za prawde</t>
+          <t xml:space="preserve">Jestem wdzieczny za prawde</t>
         </is>
       </c>
       <c r="G333" t="inlineStr">
@@ -26065,7 +26065,7 @@
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za nowe spojrzenie</t>
+          <t xml:space="preserve">Jestem wdzieczny za nowe spojrzenie</t>
         </is>
       </c>
       <c r="G334" t="inlineStr">
@@ -26143,7 +26143,7 @@
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za przyszlosc</t>
+          <t xml:space="preserve">Jestem wdzieczny za przyszlosc</t>
         </is>
       </c>
       <c r="G335" t="inlineStr">
@@ -26221,7 +26221,7 @@
       </c>
       <c r="F336" t="inlineStr">
         <is>
-          <t xml:space="preserve">Wdziecznosc za terazniejszosc</t>
+          <t xml:space="preserve">Jestem wdzieczny za terazniejszosc</t>
         </is>
       </c>
       <c r="G336" t="inlineStr">
@@ -26299,7 +26299,7 @@
       </c>
       <c r="F337" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dac to, co dostalem</t>
+          <t xml:space="preserve">Przekazuje dalej to, co sam otrzymuje</t>
         </is>
       </c>
       <c r="G337" t="inlineStr">
@@ -26377,7 +26377,7 @@
       </c>
       <c r="F338" t="inlineStr">
         <is>
-          <t xml:space="preserve">Obecnosc tez jest darem</t>
+          <t xml:space="preserve">Wiem, ze moja obecnosc tez jest darem</t>
         </is>
       </c>
       <c r="G338" t="inlineStr">
@@ -26455,7 +26455,7 @@
       </c>
       <c r="F339" t="inlineStr">
         <is>
-          <t xml:space="preserve">Sluchac zamiast pouczac</t>
+          <t xml:space="preserve">Slucham zamiast pouczac</t>
         </is>
       </c>
       <c r="G339" t="inlineStr">
@@ -26533,7 +26533,7 @@
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t xml:space="preserve">Opowiedziec prawde o swojej drodze</t>
+          <t xml:space="preserve">Opowiadam prawde o swojej drodze</t>
         </is>
       </c>
       <c r="G340" t="inlineStr">
@@ -26611,7 +26611,7 @@
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zadzwonic do kogos, kto moze potrzebowac glosu</t>
+          <t xml:space="preserve">Dzwonie do kogos, kto moze potrzebowac glosu</t>
         </is>
       </c>
       <c r="G341" t="inlineStr">
@@ -26689,7 +26689,7 @@
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie nadzieja, nie presja</t>
+          <t xml:space="preserve">Dziele sie nadzieja, nie presja</t>
         </is>
       </c>
       <c r="G342" t="inlineStr">
@@ -26767,7 +26767,7 @@
       </c>
       <c r="F343" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie spokojem</t>
+          <t xml:space="preserve">Dziele sie spokojem</t>
         </is>
       </c>
       <c r="G343" t="inlineStr">
@@ -26845,7 +26845,7 @@
       </c>
       <c r="F344" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie uwaga</t>
+          <t xml:space="preserve">Dziele sie uwaga</t>
         </is>
       </c>
       <c r="G344" t="inlineStr">
@@ -26923,7 +26923,7 @@
       </c>
       <c r="F345" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie czasem</t>
+          <t xml:space="preserve">Dziele sie czasem</t>
         </is>
       </c>
       <c r="G345" t="inlineStr">
@@ -27001,7 +27001,7 @@
       </c>
       <c r="F346" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie doswiadczeniem kryzysu i powrotu</t>
+          <t xml:space="preserve">Dziele sie doswiadczeniem kryzysu i powrotu</t>
         </is>
       </c>
       <c r="G346" t="inlineStr">
@@ -27079,7 +27079,7 @@
       </c>
       <c r="F347" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie tym, co dziala</t>
+          <t xml:space="preserve">Dziele sie tym, co dziala</t>
         </is>
       </c>
       <c r="G347" t="inlineStr">
@@ -27157,7 +27157,7 @@
       </c>
       <c r="F348" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie bez udawania mocnego</t>
+          <t xml:space="preserve">Dziele sie bez udawania mocnego</t>
         </is>
       </c>
       <c r="G348" t="inlineStr">
@@ -27235,7 +27235,7 @@
       </c>
       <c r="F349" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie wlasna kruchoscia</t>
+          <t xml:space="preserve">Dziele sie wlasna kruchoscia</t>
         </is>
       </c>
       <c r="G349" t="inlineStr">
@@ -27313,7 +27313,7 @@
       </c>
       <c r="F350" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie wdziecznoscia</t>
+          <t xml:space="preserve">Dziele sie wdziecznoscia</t>
         </is>
       </c>
       <c r="G350" t="inlineStr">
@@ -27391,7 +27391,7 @@
       </c>
       <c r="F351" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie wspolnota</t>
+          <t xml:space="preserve">Dziele sie wspolnota</t>
         </is>
       </c>
       <c r="G351" t="inlineStr">
@@ -27469,7 +27469,7 @@
       </c>
       <c r="F352" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie slowem otuchy</t>
+          <t xml:space="preserve">Dziele sie slowem otuchy</t>
         </is>
       </c>
       <c r="G352" t="inlineStr">
@@ -27547,7 +27547,7 @@
       </c>
       <c r="F353" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie obecnoscia przy trudnym dniu</t>
+          <t xml:space="preserve">Dziele sie obecnoscia przy trudnym dniu</t>
         </is>
       </c>
       <c r="G353" t="inlineStr">
@@ -27625,7 +27625,7 @@
       </c>
       <c r="F354" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie odpowiedzialnoscia</t>
+          <t xml:space="preserve">Dziele sie odpowiedzialnoscia</t>
         </is>
       </c>
       <c r="G354" t="inlineStr">
@@ -27703,7 +27703,7 @@
       </c>
       <c r="F355" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie dobrem w malej formie</t>
+          <t xml:space="preserve">Dziele sie dobrem w malej formie</t>
         </is>
       </c>
       <c r="G355" t="inlineStr">
@@ -27781,7 +27781,7 @@
       </c>
       <c r="F356" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie cierpliwoscia</t>
+          <t xml:space="preserve">Dziele sie cierpliwoscia</t>
         </is>
       </c>
       <c r="G356" t="inlineStr">
@@ -27859,7 +27859,7 @@
       </c>
       <c r="F357" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie tym, co sam chcialem uslyszec</t>
+          <t xml:space="preserve">Dziele sie tym, co sam chcialbym uslyszec</t>
         </is>
       </c>
       <c r="G357" t="inlineStr">
@@ -27937,7 +27937,7 @@
       </c>
       <c r="F358" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie w prawdzie</t>
+          <t xml:space="preserve">Dziele sie w prawdzie</t>
         </is>
       </c>
       <c r="G358" t="inlineStr">
@@ -28015,7 +28015,7 @@
       </c>
       <c r="F359" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie, nie ratujac</t>
+          <t xml:space="preserve">Dziele sie, nie ratujac</t>
         </is>
       </c>
       <c r="G359" t="inlineStr">
@@ -28093,7 +28093,7 @@
       </c>
       <c r="F360" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie pokojem</t>
+          <t xml:space="preserve">Dziele sie pokojem</t>
         </is>
       </c>
       <c r="G360" t="inlineStr">
@@ -28171,7 +28171,7 @@
       </c>
       <c r="F361" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie swiatlem</t>
+          <t xml:space="preserve">Dziele sie swiatlem</t>
         </is>
       </c>
       <c r="G361" t="inlineStr">
@@ -28249,7 +28249,7 @@
       </c>
       <c r="F362" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie nadzieja po ciemnym czasie</t>
+          <t xml:space="preserve">Dziele sie nadzieja po ciemnym czasie</t>
         </is>
       </c>
       <c r="G362" t="inlineStr">
@@ -28327,7 +28327,7 @@
       </c>
       <c r="F363" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie sensem</t>
+          <t xml:space="preserve">Dziele sie sensem</t>
         </is>
       </c>
       <c r="G363" t="inlineStr">
@@ -28405,7 +28405,7 @@
       </c>
       <c r="F364" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie droga zdrowienia</t>
+          <t xml:space="preserve">Dziele sie droga zdrowienia</t>
         </is>
       </c>
       <c r="G364" t="inlineStr">
@@ -28483,7 +28483,7 @@
       </c>
       <c r="F365" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie zyciem codziennym</t>
+          <t xml:space="preserve">Dziele sie zyciem codziennym</t>
         </is>
       </c>
       <c r="G365" t="inlineStr">
@@ -28561,7 +28561,7 @@
       </c>
       <c r="F366" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie tym, co najprostsze</t>
+          <t xml:space="preserve">Dziele sie tym, co najprostsze</t>
         </is>
       </c>
       <c r="G366" t="inlineStr">
@@ -28639,7 +28639,7 @@
       </c>
       <c r="F367" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzielic sie zyciem</t>
+          <t xml:space="preserve">Dziele sie zyciem</t>
         </is>
       </c>
       <c r="G367" t="inlineStr">
@@ -28844,7 +28844,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dzis zatrzymaj sie przy jednej rzeczy: [mysl przewodnia].</t>
+          <t xml:space="preserve">Dzis zatrzymuje sie przy jednej rzeczy: [mysl przewodnia].</t>
         </is>
       </c>
     </row>
@@ -28868,7 +28868,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Zapytaj siebie: [jedno krotkie pytanie].</t>
+          <t xml:space="preserve">Pytam siebie: [jedno krotkie pytanie].</t>
         </is>
       </c>
     </row>
@@ -28880,7 +28880,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Na dzis wystarczy jeden krok: [jedno konkretne dzialanie].</t>
+          <t xml:space="preserve">Na dzis wystarczy mi jeden krok: [jedno konkretne dzialanie].</t>
         </is>
       </c>
     </row>

</xml_diff>